<commit_message>
dataset MHD --num-walks 50 --walk-length 15 --p 2 --q 1
The results of MHD with dataset MHD --num-walks 50 --walk-length 15 --p 2 --q 1 and discarding the type in create graph, was not good
</commit_message>
<xml_diff>
--- a/results/MHD/deepwalk_embedding_size_results.xlsx
+++ b/results/MHD/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8400670257509418</v>
+        <v>0.8418291976037814</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8348779218304363</v>
+        <v>0.8327714310872041</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8276032380888587</v>
+        <v>0.8269066012482021</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8262959114278485</v>
+        <v>0.8135793022418166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run MHD --num-walks 80 --walk-length 15 --p 3 --q 1
</commit_message>
<xml_diff>
--- a/results/MHD/deepwalk_embedding_size_results.xlsx
+++ b/results/MHD/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8418291976037814</v>
+        <v>0.8393653025565531</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8327714310872041</v>
+        <v>0.836587358885196</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8269066012482021</v>
+        <v>0.8311404989383833</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8135793022418166</v>
+        <v>0.8258164652152228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MHD --num-walks 80 --walk-length 20 --p 3 --q 1
</commit_message>
<xml_diff>
--- a/results/MHD/deepwalk_embedding_size_results.xlsx
+++ b/results/MHD/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8393653025565531</v>
+        <v>0.8375663760320837</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.836587358885196</v>
+        <v>0.8374639015300185</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8311404989383833</v>
+        <v>0.8284457119535965</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8258164652152228</v>
+        <v>0.8256629086318024</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Using kNN for graph creation
</commit_message>
<xml_diff>
--- a/results/MHD/deepwalk_embedding_size_results.xlsx
+++ b/results/MHD/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8375663760320837</v>
+        <v>0.842528554246547</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8374639015300185</v>
+        <v>0.8331078590718223</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8284457119535965</v>
+        <v>0.8299060904582195</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8256629086318024</v>
+        <v>0.8219693320728817</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MHD --num-walks 80 --walk-length 15 --p 3 --q 1
The results are good,  for p=1, q=1
</commit_message>
<xml_diff>
--- a/results/MHD/deepwalk_embedding_size_results.xlsx
+++ b/results/MHD/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8401628145515341</v>
+        <v>0.8366581664678689</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8297161757349139</v>
+        <v>0.8319549957522533</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8272108055971483</v>
+        <v>0.82562614198634</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8218948669883618</v>
+        <v>0.8186308458113718</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
10000 Samples of MHD, k=10
</commit_message>
<xml_diff>
--- a/results/MHD/deepwalk_embedding_size_results.xlsx
+++ b/results/MHD/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8366581664678689</v>
+        <v>0.839727365388262</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8319549957522533</v>
+        <v>0.8329931845887062</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.82562614198634</v>
+        <v>0.8340420621688711</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8186308458113718</v>
+        <v>0.8294316623482555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>